<commit_message>
update fav matric number
</commit_message>
<xml_diff>
--- a/Backend/eligible_voters.xlsx
+++ b/Backend/eligible_voters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\E-voting-system\Backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FD50289-B1DA-4C40-A01E-99C3B81C2862}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FB86D7D-5482-4EEC-B9E0-D26821DA3FF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="400" sheetId="1" r:id="rId1"/>
@@ -1936,9 +1936,6 @@
     <t>thvgger005@gmail.com</t>
   </si>
   <si>
-    <t>22N02095</t>
-  </si>
-  <si>
     <t>ADEDEJI Enoch Favour</t>
   </si>
   <si>
@@ -2678,6 +2675,9 @@
   </si>
   <si>
     <t>seunlawaladekunle@gmail.com</t>
+  </si>
+  <si>
+    <t>23N02095</t>
   </si>
 </sst>
 </file>
@@ -3553,7 +3553,7 @@
         <v>99</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -6114,43 +6114,43 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>884</v>
+      </c>
+      <c r="B6" t="s">
         <v>637</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>638</v>
-      </c>
-      <c r="C6" t="s">
-        <v>639</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>639</v>
+      </c>
+      <c r="B7" t="s">
         <v>640</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>641</v>
-      </c>
-      <c r="C7" t="s">
-        <v>642</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>642</v>
+      </c>
+      <c r="B8" t="s">
         <v>643</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>644</v>
-      </c>
-      <c r="C8" t="s">
-        <v>645</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>645</v>
+      </c>
+      <c r="B9" t="s">
         <v>646</v>
-      </c>
-      <c r="B9" t="s">
-        <v>647</v>
       </c>
       <c r="C9" t="s">
         <v>5</v>
@@ -6158,87 +6158,87 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>647</v>
+      </c>
+      <c r="B10" t="s">
         <v>648</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>649</v>
-      </c>
-      <c r="C10" t="s">
-        <v>650</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>650</v>
+      </c>
+      <c r="B11" t="s">
         <v>651</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>652</v>
-      </c>
-      <c r="C11" t="s">
-        <v>653</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>653</v>
+      </c>
+      <c r="B12" t="s">
         <v>654</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>655</v>
-      </c>
-      <c r="C12" t="s">
-        <v>656</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>656</v>
+      </c>
+      <c r="B13" t="s">
         <v>657</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>658</v>
-      </c>
-      <c r="C13" t="s">
-        <v>659</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>659</v>
+      </c>
+      <c r="B14" t="s">
         <v>660</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>661</v>
-      </c>
-      <c r="C14" t="s">
-        <v>662</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>662</v>
+      </c>
+      <c r="B15" t="s">
         <v>663</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>664</v>
-      </c>
-      <c r="C15" t="s">
-        <v>665</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>665</v>
+      </c>
+      <c r="B16" t="s">
         <v>666</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>667</v>
-      </c>
-      <c r="C16" t="s">
-        <v>668</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>668</v>
+      </c>
+      <c r="B17" t="s">
         <v>669</v>
-      </c>
-      <c r="B17" t="s">
-        <v>670</v>
       </c>
       <c r="C17" t="s">
         <v>5</v>
@@ -6246,10 +6246,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>670</v>
+      </c>
+      <c r="B18" t="s">
         <v>671</v>
-      </c>
-      <c r="B18" t="s">
-        <v>672</v>
       </c>
       <c r="C18" t="s">
         <v>5</v>
@@ -6257,21 +6257,21 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>672</v>
+      </c>
+      <c r="B19" t="s">
         <v>673</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>674</v>
-      </c>
-      <c r="C19" t="s">
-        <v>675</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>675</v>
+      </c>
+      <c r="B20" t="s">
         <v>676</v>
-      </c>
-      <c r="B20" t="s">
-        <v>677</v>
       </c>
       <c r="C20" t="s">
         <v>5</v>
@@ -6279,120 +6279,120 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>677</v>
+      </c>
+      <c r="B21" t="s">
         <v>678</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
         <v>679</v>
-      </c>
-      <c r="C21" t="s">
-        <v>680</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>680</v>
+      </c>
+      <c r="B22" t="s">
         <v>681</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
         <v>682</v>
-      </c>
-      <c r="C22" t="s">
-        <v>683</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>683</v>
+      </c>
+      <c r="B23" t="s">
         <v>684</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" t="s">
         <v>685</v>
-      </c>
-      <c r="C23" t="s">
-        <v>686</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>686</v>
+      </c>
+      <c r="B24" t="s">
         <v>687</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>688</v>
-      </c>
-      <c r="C24" t="s">
-        <v>689</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>689</v>
+      </c>
+      <c r="B25" t="s">
         <v>690</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
         <v>691</v>
-      </c>
-      <c r="C25" t="s">
-        <v>692</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>692</v>
+      </c>
+      <c r="B26" t="s">
         <v>693</v>
       </c>
-      <c r="B26" t="s">
+      <c r="C26" t="s">
         <v>694</v>
-      </c>
-      <c r="C26" t="s">
-        <v>695</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>695</v>
+      </c>
+      <c r="B27" t="s">
         <v>696</v>
       </c>
-      <c r="B27" t="s">
+      <c r="C27" t="s">
         <v>697</v>
-      </c>
-      <c r="C27" t="s">
-        <v>698</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>698</v>
+      </c>
+      <c r="B28" t="s">
         <v>699</v>
       </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
         <v>700</v>
-      </c>
-      <c r="C28" t="s">
-        <v>701</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>701</v>
+      </c>
+      <c r="B29" t="s">
         <v>702</v>
       </c>
-      <c r="B29" t="s">
+      <c r="C29" t="s">
         <v>703</v>
-      </c>
-      <c r="C29" t="s">
-        <v>704</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>704</v>
+      </c>
+      <c r="B30" t="s">
         <v>705</v>
       </c>
-      <c r="B30" t="s">
+      <c r="C30" t="s">
         <v>706</v>
-      </c>
-      <c r="C30" t="s">
-        <v>707</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>707</v>
+      </c>
+      <c r="B31" t="s">
         <v>708</v>
-      </c>
-      <c r="B31" t="s">
-        <v>709</v>
       </c>
       <c r="C31" t="s">
         <v>5</v>
@@ -6400,98 +6400,98 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>709</v>
+      </c>
+      <c r="B32" t="s">
         <v>710</v>
       </c>
-      <c r="B32" t="s">
+      <c r="C32" t="s">
         <v>711</v>
-      </c>
-      <c r="C32" t="s">
-        <v>712</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>712</v>
+      </c>
+      <c r="B33" t="s">
         <v>713</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
         <v>714</v>
-      </c>
-      <c r="C33" t="s">
-        <v>715</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>715</v>
+      </c>
+      <c r="B34" t="s">
         <v>716</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" t="s">
         <v>717</v>
-      </c>
-      <c r="C34" t="s">
-        <v>718</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>718</v>
+      </c>
+      <c r="B35" t="s">
         <v>719</v>
       </c>
-      <c r="B35" t="s">
+      <c r="C35" t="s">
         <v>720</v>
-      </c>
-      <c r="C35" t="s">
-        <v>721</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>721</v>
+      </c>
+      <c r="B36" t="s">
         <v>722</v>
       </c>
-      <c r="B36" t="s">
+      <c r="C36" t="s">
         <v>723</v>
-      </c>
-      <c r="C36" t="s">
-        <v>724</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>724</v>
+      </c>
+      <c r="B37" t="s">
         <v>725</v>
       </c>
-      <c r="B37" t="s">
+      <c r="C37" t="s">
         <v>726</v>
-      </c>
-      <c r="C37" t="s">
-        <v>727</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>727</v>
+      </c>
+      <c r="B38" t="s">
         <v>728</v>
       </c>
-      <c r="B38" t="s">
+      <c r="C38" t="s">
         <v>729</v>
-      </c>
-      <c r="C38" t="s">
-        <v>730</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>730</v>
+      </c>
+      <c r="B39" t="s">
         <v>731</v>
       </c>
-      <c r="B39" t="s">
+      <c r="C39" t="s">
         <v>732</v>
-      </c>
-      <c r="C39" t="s">
-        <v>733</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>733</v>
+      </c>
+      <c r="B40" t="s">
         <v>734</v>
-      </c>
-      <c r="B40" t="s">
-        <v>735</v>
       </c>
       <c r="C40" t="s">
         <v>5</v>
@@ -6499,10 +6499,10 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>735</v>
+      </c>
+      <c r="B41" t="s">
         <v>736</v>
-      </c>
-      <c r="B41" t="s">
-        <v>737</v>
       </c>
       <c r="C41" t="s">
         <v>5</v>
@@ -6510,285 +6510,285 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>737</v>
+      </c>
+      <c r="B42" t="s">
         <v>738</v>
       </c>
-      <c r="B42" t="s">
+      <c r="C42" t="s">
         <v>739</v>
-      </c>
-      <c r="C42" t="s">
-        <v>740</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>740</v>
+      </c>
+      <c r="B43" t="s">
         <v>741</v>
       </c>
-      <c r="B43" t="s">
+      <c r="C43" t="s">
         <v>742</v>
-      </c>
-      <c r="C43" t="s">
-        <v>743</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>743</v>
+      </c>
+      <c r="B44" t="s">
         <v>744</v>
       </c>
-      <c r="B44" t="s">
+      <c r="C44" t="s">
         <v>745</v>
-      </c>
-      <c r="C44" t="s">
-        <v>746</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
+        <v>746</v>
+      </c>
+      <c r="B45" t="s">
         <v>747</v>
       </c>
-      <c r="B45" t="s">
+      <c r="C45" t="s">
         <v>748</v>
-      </c>
-      <c r="C45" t="s">
-        <v>749</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>749</v>
+      </c>
+      <c r="B46" t="s">
         <v>750</v>
       </c>
-      <c r="B46" t="s">
+      <c r="C46" t="s">
         <v>751</v>
-      </c>
-      <c r="C46" t="s">
-        <v>752</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
+        <v>752</v>
+      </c>
+      <c r="B47" t="s">
         <v>753</v>
       </c>
-      <c r="B47" t="s">
+      <c r="C47" t="s">
         <v>754</v>
-      </c>
-      <c r="C47" t="s">
-        <v>755</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>755</v>
+      </c>
+      <c r="B48" t="s">
         <v>756</v>
       </c>
-      <c r="B48" t="s">
+      <c r="C48" t="s">
         <v>757</v>
-      </c>
-      <c r="C48" t="s">
-        <v>758</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>758</v>
+      </c>
+      <c r="B49" t="s">
         <v>759</v>
       </c>
-      <c r="B49" t="s">
+      <c r="C49" t="s">
         <v>760</v>
-      </c>
-      <c r="C49" t="s">
-        <v>761</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>761</v>
+      </c>
+      <c r="B50" t="s">
         <v>762</v>
       </c>
-      <c r="B50" t="s">
+      <c r="C50" t="s">
         <v>763</v>
-      </c>
-      <c r="C50" t="s">
-        <v>764</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>764</v>
+      </c>
+      <c r="B51" t="s">
         <v>765</v>
       </c>
-      <c r="B51" t="s">
+      <c r="C51" t="s">
         <v>766</v>
-      </c>
-      <c r="C51" t="s">
-        <v>767</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>767</v>
+      </c>
+      <c r="B52" t="s">
         <v>768</v>
       </c>
-      <c r="B52" t="s">
+      <c r="C52" t="s">
         <v>769</v>
-      </c>
-      <c r="C52" t="s">
-        <v>770</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>770</v>
+      </c>
+      <c r="B53" t="s">
         <v>771</v>
       </c>
-      <c r="B53" t="s">
+      <c r="C53" t="s">
         <v>772</v>
-      </c>
-      <c r="C53" t="s">
-        <v>773</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>773</v>
+      </c>
+      <c r="B54" t="s">
         <v>774</v>
       </c>
-      <c r="B54" t="s">
+      <c r="C54" t="s">
         <v>775</v>
-      </c>
-      <c r="C54" t="s">
-        <v>776</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>776</v>
+      </c>
+      <c r="B55" t="s">
         <v>777</v>
       </c>
-      <c r="B55" t="s">
+      <c r="C55" t="s">
         <v>778</v>
-      </c>
-      <c r="C55" t="s">
-        <v>779</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>779</v>
+      </c>
+      <c r="B56" t="s">
         <v>780</v>
       </c>
-      <c r="B56" t="s">
+      <c r="C56" t="s">
         <v>781</v>
-      </c>
-      <c r="C56" t="s">
-        <v>782</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
+        <v>782</v>
+      </c>
+      <c r="B57" t="s">
         <v>783</v>
       </c>
-      <c r="B57" t="s">
+      <c r="C57" t="s">
         <v>784</v>
-      </c>
-      <c r="C57" t="s">
-        <v>785</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
+        <v>785</v>
+      </c>
+      <c r="B58" t="s">
         <v>786</v>
       </c>
-      <c r="B58" t="s">
+      <c r="C58" t="s">
         <v>787</v>
-      </c>
-      <c r="C58" t="s">
-        <v>788</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
+        <v>788</v>
+      </c>
+      <c r="B59" t="s">
         <v>789</v>
       </c>
-      <c r="B59" t="s">
+      <c r="C59" t="s">
         <v>790</v>
-      </c>
-      <c r="C59" t="s">
-        <v>791</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>791</v>
+      </c>
+      <c r="B60" t="s">
         <v>792</v>
       </c>
-      <c r="B60" t="s">
+      <c r="C60" t="s">
         <v>793</v>
-      </c>
-      <c r="C60" t="s">
-        <v>794</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
+        <v>794</v>
+      </c>
+      <c r="B61" t="s">
         <v>795</v>
       </c>
-      <c r="B61" t="s">
+      <c r="C61" t="s">
         <v>796</v>
-      </c>
-      <c r="C61" t="s">
-        <v>797</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
+        <v>797</v>
+      </c>
+      <c r="B62" t="s">
         <v>798</v>
       </c>
-      <c r="B62" t="s">
+      <c r="C62" t="s">
         <v>799</v>
-      </c>
-      <c r="C62" t="s">
-        <v>800</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
+        <v>800</v>
+      </c>
+      <c r="B63" t="s">
         <v>801</v>
       </c>
-      <c r="B63" t="s">
+      <c r="C63" t="s">
         <v>802</v>
-      </c>
-      <c r="C63" t="s">
-        <v>803</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>803</v>
+      </c>
+      <c r="B64" t="s">
         <v>804</v>
       </c>
-      <c r="B64" t="s">
+      <c r="C64" t="s">
         <v>805</v>
-      </c>
-      <c r="C64" t="s">
-        <v>806</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>806</v>
+      </c>
+      <c r="B65" t="s">
         <v>807</v>
       </c>
-      <c r="B65" t="s">
+      <c r="C65" t="s">
         <v>808</v>
-      </c>
-      <c r="C65" t="s">
-        <v>809</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
+        <v>809</v>
+      </c>
+      <c r="B66" t="s">
         <v>810</v>
       </c>
-      <c r="B66" t="s">
+      <c r="C66" t="s">
         <v>811</v>
-      </c>
-      <c r="C66" t="s">
-        <v>812</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
+        <v>812</v>
+      </c>
+      <c r="B67" t="s">
         <v>813</v>
-      </c>
-      <c r="B67" t="s">
-        <v>814</v>
       </c>
       <c r="C67" t="s">
         <v>5</v>
@@ -6796,43 +6796,43 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>814</v>
+      </c>
+      <c r="B68" t="s">
         <v>815</v>
       </c>
-      <c r="B68" t="s">
+      <c r="C68" t="s">
         <v>816</v>
-      </c>
-      <c r="C68" t="s">
-        <v>817</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
+        <v>817</v>
+      </c>
+      <c r="B69" t="s">
         <v>818</v>
       </c>
-      <c r="B69" t="s">
+      <c r="C69" t="s">
         <v>819</v>
-      </c>
-      <c r="C69" t="s">
-        <v>820</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>820</v>
+      </c>
+      <c r="B70" t="s">
         <v>821</v>
       </c>
-      <c r="B70" t="s">
+      <c r="C70" t="s">
         <v>822</v>
-      </c>
-      <c r="C70" t="s">
-        <v>823</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
+        <v>823</v>
+      </c>
+      <c r="B71" t="s">
         <v>824</v>
-      </c>
-      <c r="B71" t="s">
-        <v>825</v>
       </c>
       <c r="C71" t="s">
         <v>5</v>
@@ -6840,10 +6840,10 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
+        <v>825</v>
+      </c>
+      <c r="B72" t="s">
         <v>826</v>
-      </c>
-      <c r="B72" t="s">
-        <v>827</v>
       </c>
       <c r="C72" t="s">
         <v>5</v>
@@ -6851,10 +6851,10 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
+        <v>827</v>
+      </c>
+      <c r="B73" t="s">
         <v>828</v>
-      </c>
-      <c r="B73" t="s">
-        <v>829</v>
       </c>
       <c r="C73" t="s">
         <v>5</v>
@@ -6865,7 +6865,7 @@
         <v>271</v>
       </c>
       <c r="B74" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="C74" t="s">
         <v>273</v>
@@ -6873,10 +6873,10 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
+        <v>830</v>
+      </c>
+      <c r="B75" t="s">
         <v>831</v>
-      </c>
-      <c r="B75" t="s">
-        <v>832</v>
       </c>
       <c r="C75" t="s">
         <v>5</v>
@@ -6884,43 +6884,43 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
+        <v>832</v>
+      </c>
+      <c r="B76" t="s">
         <v>833</v>
       </c>
-      <c r="B76" t="s">
+      <c r="C76" t="s">
         <v>834</v>
-      </c>
-      <c r="C76" t="s">
-        <v>835</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
+        <v>835</v>
+      </c>
+      <c r="B77" t="s">
         <v>836</v>
       </c>
-      <c r="B77" t="s">
+      <c r="C77" t="s">
         <v>837</v>
-      </c>
-      <c r="C77" t="s">
-        <v>838</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
+        <v>838</v>
+      </c>
+      <c r="B78" t="s">
         <v>839</v>
       </c>
-      <c r="B78" t="s">
+      <c r="C78" t="s">
         <v>840</v>
-      </c>
-      <c r="C78" t="s">
-        <v>841</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
+        <v>841</v>
+      </c>
+      <c r="B79" t="s">
         <v>842</v>
-      </c>
-      <c r="B79" t="s">
-        <v>843</v>
       </c>
       <c r="C79" t="s">
         <v>5</v>
@@ -6928,21 +6928,21 @@
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
+        <v>843</v>
+      </c>
+      <c r="B80" t="s">
         <v>844</v>
       </c>
-      <c r="B80" t="s">
+      <c r="C80" t="s">
         <v>845</v>
-      </c>
-      <c r="C80" t="s">
-        <v>846</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
+        <v>846</v>
+      </c>
+      <c r="B81" t="s">
         <v>847</v>
-      </c>
-      <c r="B81" t="s">
-        <v>848</v>
       </c>
       <c r="C81" t="s">
         <v>5</v>
@@ -6950,21 +6950,21 @@
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>848</v>
+      </c>
+      <c r="B82" t="s">
         <v>849</v>
       </c>
-      <c r="B82" t="s">
+      <c r="C82" t="s">
         <v>850</v>
-      </c>
-      <c r="C82" t="s">
-        <v>851</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
+        <v>851</v>
+      </c>
+      <c r="B83" t="s">
         <v>852</v>
-      </c>
-      <c r="B83" t="s">
-        <v>853</v>
       </c>
       <c r="C83" t="s">
         <v>5</v>
@@ -6972,21 +6972,21 @@
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
+        <v>853</v>
+      </c>
+      <c r="B84" t="s">
         <v>854</v>
       </c>
-      <c r="B84" t="s">
+      <c r="C84" t="s">
         <v>855</v>
-      </c>
-      <c r="C84" t="s">
-        <v>856</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
+        <v>856</v>
+      </c>
+      <c r="B85" t="s">
         <v>857</v>
-      </c>
-      <c r="B85" t="s">
-        <v>858</v>
       </c>
       <c r="C85" t="s">
         <v>5</v>
@@ -6994,10 +6994,10 @@
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
+        <v>858</v>
+      </c>
+      <c r="B86" t="s">
         <v>859</v>
-      </c>
-      <c r="B86" t="s">
-        <v>860</v>
       </c>
       <c r="C86" t="s">
         <v>5</v>
@@ -7005,79 +7005,79 @@
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
+        <v>860</v>
+      </c>
+      <c r="B87" t="s">
         <v>861</v>
       </c>
-      <c r="B87" t="s">
+      <c r="C87" t="s">
         <v>862</v>
-      </c>
-      <c r="C87" t="s">
-        <v>863</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="B88" t="s">
+        <v>673</v>
+      </c>
+      <c r="C88" t="s">
         <v>674</v>
-      </c>
-      <c r="C88" t="s">
-        <v>675</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
+        <v>864</v>
+      </c>
+      <c r="B89" t="s">
         <v>865</v>
       </c>
-      <c r="B89" t="s">
+      <c r="C89" t="s">
         <v>866</v>
-      </c>
-      <c r="C89" t="s">
-        <v>867</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
+        <v>867</v>
+      </c>
+      <c r="B90" t="s">
         <v>868</v>
       </c>
-      <c r="B90" t="s">
+      <c r="C90" t="s">
         <v>869</v>
-      </c>
-      <c r="C90" t="s">
-        <v>870</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
+        <v>870</v>
+      </c>
+      <c r="B91" t="s">
         <v>871</v>
       </c>
-      <c r="B91" t="s">
+      <c r="C91" t="s">
         <v>872</v>
-      </c>
-      <c r="C91" t="s">
-        <v>873</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
+        <v>873</v>
+      </c>
+      <c r="B92" t="s">
         <v>874</v>
       </c>
-      <c r="B92" t="s">
+      <c r="C92" t="s">
         <v>875</v>
-      </c>
-      <c r="C92" t="s">
-        <v>876</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
+        <v>876</v>
+      </c>
+      <c r="B93" t="s">
         <v>877</v>
       </c>
-      <c r="B93" t="s">
+      <c r="C93" t="s">
         <v>878</v>
-      </c>
-      <c r="C93" t="s">
-        <v>879</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
@@ -7085,27 +7085,27 @@
         <v>267</v>
       </c>
       <c r="B94" t="s">
+        <v>879</v>
+      </c>
+      <c r="C94" t="s">
         <v>880</v>
-      </c>
-      <c r="C94" t="s">
-        <v>881</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="B95" t="s">
+        <v>881</v>
+      </c>
+      <c r="C95" t="s">
         <v>882</v>
-      </c>
-      <c r="C95" t="s">
-        <v>883</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:C95" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:C5 A7:C95 B6:C6" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated praise 300 level record
</commit_message>
<xml_diff>
--- a/Backend/eligible_voters.xlsx
+++ b/Backend/eligible_voters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\E-voting-system\Backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FB86D7D-5482-4EEC-B9E0-D26821DA3FF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF6AA3DD-FD8B-47D9-939B-F878A0D3CA16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="400" sheetId="1" r:id="rId1"/>
@@ -2293,12 +2293,6 @@
     <t>23N02067</t>
   </si>
   <si>
-    <t>OLANPEJU Ayomide Praise</t>
-  </si>
-  <si>
-    <t>ayomdiepraize2007@gmail.com</t>
-  </si>
-  <si>
     <t>23N02068</t>
   </si>
   <si>
@@ -2678,6 +2672,12 @@
   </si>
   <si>
     <t>23N02095</t>
+  </si>
+  <si>
+    <t>OLANPEJO Ayomide Praise</t>
+  </si>
+  <si>
+    <t>ayomidepraize2007@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -3553,7 +3553,7 @@
         <v>99</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>883</v>
+        <v>881</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -6114,7 +6114,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>884</v>
+        <v>882</v>
       </c>
       <c r="B6" t="s">
         <v>637</v>
@@ -6579,216 +6579,216 @@
         <v>755</v>
       </c>
       <c r="B48" t="s">
-        <v>756</v>
-      </c>
-      <c r="C48" t="s">
-        <v>757</v>
+        <v>883</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>884</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>756</v>
+      </c>
+      <c r="B49" t="s">
+        <v>757</v>
+      </c>
+      <c r="C49" t="s">
         <v>758</v>
-      </c>
-      <c r="B49" t="s">
-        <v>759</v>
-      </c>
-      <c r="C49" t="s">
-        <v>760</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>759</v>
+      </c>
+      <c r="B50" t="s">
+        <v>760</v>
+      </c>
+      <c r="C50" t="s">
         <v>761</v>
-      </c>
-      <c r="B50" t="s">
-        <v>762</v>
-      </c>
-      <c r="C50" t="s">
-        <v>763</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>762</v>
+      </c>
+      <c r="B51" t="s">
+        <v>763</v>
+      </c>
+      <c r="C51" t="s">
         <v>764</v>
-      </c>
-      <c r="B51" t="s">
-        <v>765</v>
-      </c>
-      <c r="C51" t="s">
-        <v>766</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>765</v>
+      </c>
+      <c r="B52" t="s">
+        <v>766</v>
+      </c>
+      <c r="C52" t="s">
         <v>767</v>
-      </c>
-      <c r="B52" t="s">
-        <v>768</v>
-      </c>
-      <c r="C52" t="s">
-        <v>769</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>768</v>
+      </c>
+      <c r="B53" t="s">
+        <v>769</v>
+      </c>
+      <c r="C53" t="s">
         <v>770</v>
-      </c>
-      <c r="B53" t="s">
-        <v>771</v>
-      </c>
-      <c r="C53" t="s">
-        <v>772</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>771</v>
+      </c>
+      <c r="B54" t="s">
+        <v>772</v>
+      </c>
+      <c r="C54" t="s">
         <v>773</v>
-      </c>
-      <c r="B54" t="s">
-        <v>774</v>
-      </c>
-      <c r="C54" t="s">
-        <v>775</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>774</v>
+      </c>
+      <c r="B55" t="s">
+        <v>775</v>
+      </c>
+      <c r="C55" t="s">
         <v>776</v>
-      </c>
-      <c r="B55" t="s">
-        <v>777</v>
-      </c>
-      <c r="C55" t="s">
-        <v>778</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>777</v>
+      </c>
+      <c r="B56" t="s">
+        <v>778</v>
+      </c>
+      <c r="C56" t="s">
         <v>779</v>
-      </c>
-      <c r="B56" t="s">
-        <v>780</v>
-      </c>
-      <c r="C56" t="s">
-        <v>781</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
+        <v>780</v>
+      </c>
+      <c r="B57" t="s">
+        <v>781</v>
+      </c>
+      <c r="C57" t="s">
         <v>782</v>
-      </c>
-      <c r="B57" t="s">
-        <v>783</v>
-      </c>
-      <c r="C57" t="s">
-        <v>784</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
+        <v>783</v>
+      </c>
+      <c r="B58" t="s">
+        <v>784</v>
+      </c>
+      <c r="C58" t="s">
         <v>785</v>
-      </c>
-      <c r="B58" t="s">
-        <v>786</v>
-      </c>
-      <c r="C58" t="s">
-        <v>787</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
+        <v>786</v>
+      </c>
+      <c r="B59" t="s">
+        <v>787</v>
+      </c>
+      <c r="C59" t="s">
         <v>788</v>
-      </c>
-      <c r="B59" t="s">
-        <v>789</v>
-      </c>
-      <c r="C59" t="s">
-        <v>790</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>789</v>
+      </c>
+      <c r="B60" t="s">
+        <v>790</v>
+      </c>
+      <c r="C60" t="s">
         <v>791</v>
-      </c>
-      <c r="B60" t="s">
-        <v>792</v>
-      </c>
-      <c r="C60" t="s">
-        <v>793</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
+        <v>792</v>
+      </c>
+      <c r="B61" t="s">
+        <v>793</v>
+      </c>
+      <c r="C61" t="s">
         <v>794</v>
-      </c>
-      <c r="B61" t="s">
-        <v>795</v>
-      </c>
-      <c r="C61" t="s">
-        <v>796</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
+        <v>795</v>
+      </c>
+      <c r="B62" t="s">
+        <v>796</v>
+      </c>
+      <c r="C62" t="s">
         <v>797</v>
-      </c>
-      <c r="B62" t="s">
-        <v>798</v>
-      </c>
-      <c r="C62" t="s">
-        <v>799</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
+        <v>798</v>
+      </c>
+      <c r="B63" t="s">
+        <v>799</v>
+      </c>
+      <c r="C63" t="s">
         <v>800</v>
-      </c>
-      <c r="B63" t="s">
-        <v>801</v>
-      </c>
-      <c r="C63" t="s">
-        <v>802</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>801</v>
+      </c>
+      <c r="B64" t="s">
+        <v>802</v>
+      </c>
+      <c r="C64" t="s">
         <v>803</v>
-      </c>
-      <c r="B64" t="s">
-        <v>804</v>
-      </c>
-      <c r="C64" t="s">
-        <v>805</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>804</v>
+      </c>
+      <c r="B65" t="s">
+        <v>805</v>
+      </c>
+      <c r="C65" t="s">
         <v>806</v>
-      </c>
-      <c r="B65" t="s">
-        <v>807</v>
-      </c>
-      <c r="C65" t="s">
-        <v>808</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
+        <v>807</v>
+      </c>
+      <c r="B66" t="s">
+        <v>808</v>
+      </c>
+      <c r="C66" t="s">
         <v>809</v>
-      </c>
-      <c r="B66" t="s">
-        <v>810</v>
-      </c>
-      <c r="C66" t="s">
-        <v>811</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>812</v>
+        <v>810</v>
       </c>
       <c r="B67" t="s">
-        <v>813</v>
+        <v>811</v>
       </c>
       <c r="C67" t="s">
         <v>5</v>
@@ -6796,43 +6796,43 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>812</v>
+      </c>
+      <c r="B68" t="s">
+        <v>813</v>
+      </c>
+      <c r="C68" t="s">
         <v>814</v>
-      </c>
-      <c r="B68" t="s">
-        <v>815</v>
-      </c>
-      <c r="C68" t="s">
-        <v>816</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
+        <v>815</v>
+      </c>
+      <c r="B69" t="s">
+        <v>816</v>
+      </c>
+      <c r="C69" t="s">
         <v>817</v>
-      </c>
-      <c r="B69" t="s">
-        <v>818</v>
-      </c>
-      <c r="C69" t="s">
-        <v>819</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>818</v>
+      </c>
+      <c r="B70" t="s">
+        <v>819</v>
+      </c>
+      <c r="C70" t="s">
         <v>820</v>
-      </c>
-      <c r="B70" t="s">
-        <v>821</v>
-      </c>
-      <c r="C70" t="s">
-        <v>822</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>823</v>
+        <v>821</v>
       </c>
       <c r="B71" t="s">
-        <v>824</v>
+        <v>822</v>
       </c>
       <c r="C71" t="s">
         <v>5</v>
@@ -6840,10 +6840,10 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>825</v>
+        <v>823</v>
       </c>
       <c r="B72" t="s">
-        <v>826</v>
+        <v>824</v>
       </c>
       <c r="C72" t="s">
         <v>5</v>
@@ -6851,10 +6851,10 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>827</v>
+        <v>825</v>
       </c>
       <c r="B73" t="s">
-        <v>828</v>
+        <v>826</v>
       </c>
       <c r="C73" t="s">
         <v>5</v>
@@ -6865,7 +6865,7 @@
         <v>271</v>
       </c>
       <c r="B74" t="s">
-        <v>829</v>
+        <v>827</v>
       </c>
       <c r="C74" t="s">
         <v>273</v>
@@ -6873,10 +6873,10 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>830</v>
+        <v>828</v>
       </c>
       <c r="B75" t="s">
-        <v>831</v>
+        <v>829</v>
       </c>
       <c r="C75" t="s">
         <v>5</v>
@@ -6884,43 +6884,43 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
+        <v>830</v>
+      </c>
+      <c r="B76" t="s">
+        <v>831</v>
+      </c>
+      <c r="C76" t="s">
         <v>832</v>
-      </c>
-      <c r="B76" t="s">
-        <v>833</v>
-      </c>
-      <c r="C76" t="s">
-        <v>834</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
+        <v>833</v>
+      </c>
+      <c r="B77" t="s">
+        <v>834</v>
+      </c>
+      <c r="C77" t="s">
         <v>835</v>
-      </c>
-      <c r="B77" t="s">
-        <v>836</v>
-      </c>
-      <c r="C77" t="s">
-        <v>837</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
+        <v>836</v>
+      </c>
+      <c r="B78" t="s">
+        <v>837</v>
+      </c>
+      <c r="C78" t="s">
         <v>838</v>
-      </c>
-      <c r="B78" t="s">
-        <v>839</v>
-      </c>
-      <c r="C78" t="s">
-        <v>840</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>841</v>
+        <v>839</v>
       </c>
       <c r="B79" t="s">
-        <v>842</v>
+        <v>840</v>
       </c>
       <c r="C79" t="s">
         <v>5</v>
@@ -6928,21 +6928,21 @@
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
+        <v>841</v>
+      </c>
+      <c r="B80" t="s">
+        <v>842</v>
+      </c>
+      <c r="C80" t="s">
         <v>843</v>
-      </c>
-      <c r="B80" t="s">
-        <v>844</v>
-      </c>
-      <c r="C80" t="s">
-        <v>845</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>846</v>
+        <v>844</v>
       </c>
       <c r="B81" t="s">
-        <v>847</v>
+        <v>845</v>
       </c>
       <c r="C81" t="s">
         <v>5</v>
@@ -6950,21 +6950,21 @@
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>846</v>
+      </c>
+      <c r="B82" t="s">
+        <v>847</v>
+      </c>
+      <c r="C82" t="s">
         <v>848</v>
-      </c>
-      <c r="B82" t="s">
-        <v>849</v>
-      </c>
-      <c r="C82" t="s">
-        <v>850</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>851</v>
+        <v>849</v>
       </c>
       <c r="B83" t="s">
-        <v>852</v>
+        <v>850</v>
       </c>
       <c r="C83" t="s">
         <v>5</v>
@@ -6972,21 +6972,21 @@
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
+        <v>851</v>
+      </c>
+      <c r="B84" t="s">
+        <v>852</v>
+      </c>
+      <c r="C84" t="s">
         <v>853</v>
-      </c>
-      <c r="B84" t="s">
-        <v>854</v>
-      </c>
-      <c r="C84" t="s">
-        <v>855</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>856</v>
+        <v>854</v>
       </c>
       <c r="B85" t="s">
-        <v>857</v>
+        <v>855</v>
       </c>
       <c r="C85" t="s">
         <v>5</v>
@@ -6994,10 +6994,10 @@
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>858</v>
+        <v>856</v>
       </c>
       <c r="B86" t="s">
-        <v>859</v>
+        <v>857</v>
       </c>
       <c r="C86" t="s">
         <v>5</v>
@@ -7005,18 +7005,18 @@
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
+        <v>858</v>
+      </c>
+      <c r="B87" t="s">
+        <v>859</v>
+      </c>
+      <c r="C87" t="s">
         <v>860</v>
-      </c>
-      <c r="B87" t="s">
-        <v>861</v>
-      </c>
-      <c r="C87" t="s">
-        <v>862</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
       <c r="B88" t="s">
         <v>673</v>
@@ -7027,57 +7027,57 @@
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
+        <v>862</v>
+      </c>
+      <c r="B89" t="s">
+        <v>863</v>
+      </c>
+      <c r="C89" t="s">
         <v>864</v>
-      </c>
-      <c r="B89" t="s">
-        <v>865</v>
-      </c>
-      <c r="C89" t="s">
-        <v>866</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
+        <v>865</v>
+      </c>
+      <c r="B90" t="s">
+        <v>866</v>
+      </c>
+      <c r="C90" t="s">
         <v>867</v>
-      </c>
-      <c r="B90" t="s">
-        <v>868</v>
-      </c>
-      <c r="C90" t="s">
-        <v>869</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
+        <v>868</v>
+      </c>
+      <c r="B91" t="s">
+        <v>869</v>
+      </c>
+      <c r="C91" t="s">
         <v>870</v>
-      </c>
-      <c r="B91" t="s">
-        <v>871</v>
-      </c>
-      <c r="C91" t="s">
-        <v>872</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
+        <v>871</v>
+      </c>
+      <c r="B92" t="s">
+        <v>872</v>
+      </c>
+      <c r="C92" t="s">
         <v>873</v>
-      </c>
-      <c r="B92" t="s">
-        <v>874</v>
-      </c>
-      <c r="C92" t="s">
-        <v>875</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
+        <v>874</v>
+      </c>
+      <c r="B93" t="s">
+        <v>875</v>
+      </c>
+      <c r="C93" t="s">
         <v>876</v>
-      </c>
-      <c r="B93" t="s">
-        <v>877</v>
-      </c>
-      <c r="C93" t="s">
-        <v>878</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
@@ -7085,27 +7085,30 @@
         <v>267</v>
       </c>
       <c r="B94" t="s">
-        <v>879</v>
+        <v>877</v>
       </c>
       <c r="C94" t="s">
-        <v>880</v>
+        <v>878</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
       <c r="B95" t="s">
-        <v>881</v>
+        <v>879</v>
       </c>
       <c r="C95" t="s">
-        <v>882</v>
+        <v>880</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C48" r:id="rId1" xr:uid="{39895FA7-0FDE-492B-97E9-922415E968B4}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:C5 A7:C95 B6:C6" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:C5 A7:C47 B6:C6 A49:C95 A48" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: update eligible voters data file
</commit_message>
<xml_diff>
--- a/Backend/eligible_voters.xlsx
+++ b/Backend/eligible_voters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\E-voting-system\Backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF6AA3DD-FD8B-47D9-939B-F878A0D3CA16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22C7A54E-D16B-4F9D-8A9C-FE32B792B20E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="400" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1094" uniqueCount="885">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1091" uniqueCount="885">
   <si>
     <t>Matric Number</t>
   </si>
@@ -1402,9 +1402,6 @@
     <t>adelekemalik111@gmail.com</t>
   </si>
   <si>
-    <t>24NO2069</t>
-  </si>
-  <si>
     <t>ONABANJO GABRIEL JOMILOJU</t>
   </si>
   <si>
@@ -2678,6 +2675,9 @@
   </si>
   <si>
     <t>ayomidepraize2007@gmail.com</t>
+  </si>
+  <si>
+    <t>ACU20262780</t>
   </si>
 </sst>
 </file>
@@ -3553,7 +3553,7 @@
         <v>99</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -5048,17 +5048,6 @@
         <v>5</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>421</v>
-      </c>
-      <c r="B58" t="s">
-        <v>5</v>
-      </c>
-      <c r="C58" t="s">
-        <v>5</v>
-      </c>
-    </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>422</v>
@@ -5204,13 +5193,13 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
+        <v>421</v>
+      </c>
+      <c r="B72" t="s">
         <v>459</v>
       </c>
-      <c r="B72" t="s">
+      <c r="C72" t="s">
         <v>460</v>
-      </c>
-      <c r="C72" t="s">
-        <v>461</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
@@ -5218,16 +5207,16 @@
         <v>401</v>
       </c>
       <c r="B73" t="s">
+        <v>461</v>
+      </c>
+      <c r="C73" t="s">
         <v>462</v>
-      </c>
-      <c r="C73" t="s">
-        <v>463</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:C73" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:C57 A59:C71 A73:C73 B72:C72" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5250,7 +5239,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
@@ -5258,38 +5247,38 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>464</v>
+      </c>
+      <c r="B2" t="s">
         <v>465</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>466</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>467</v>
-      </c>
-      <c r="D2" t="s">
-        <v>468</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>468</v>
+      </c>
+      <c r="B3" t="s">
         <v>469</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>470</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>471</v>
-      </c>
-      <c r="D3" t="s">
-        <v>472</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>472</v>
+      </c>
+      <c r="B4" t="s">
         <v>473</v>
-      </c>
-      <c r="B4" t="s">
-        <v>474</v>
       </c>
       <c r="C4" t="s">
         <v>5</v>
@@ -5300,10 +5289,10 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>474</v>
+      </c>
+      <c r="B5" t="s">
         <v>475</v>
-      </c>
-      <c r="B5" t="s">
-        <v>476</v>
       </c>
       <c r="C5" t="s">
         <v>5</v>
@@ -5314,66 +5303,66 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>476</v>
+      </c>
+      <c r="B6" t="s">
         <v>477</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>478</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>479</v>
-      </c>
-      <c r="D6" t="s">
-        <v>480</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>480</v>
+      </c>
+      <c r="B7" t="s">
         <v>481</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>482</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>483</v>
-      </c>
-      <c r="D7" t="s">
-        <v>484</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>484</v>
+      </c>
+      <c r="B8" t="s">
         <v>485</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>486</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>487</v>
-      </c>
-      <c r="D8" t="s">
-        <v>488</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>488</v>
+      </c>
+      <c r="B9" t="s">
         <v>489</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>490</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>491</v>
-      </c>
-      <c r="D9" t="s">
-        <v>492</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>492</v>
+      </c>
+      <c r="B10" t="s">
         <v>493</v>
-      </c>
-      <c r="B10" t="s">
-        <v>494</v>
       </c>
       <c r="C10" t="s">
         <v>5</v>
@@ -5384,10 +5373,10 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>494</v>
+      </c>
+      <c r="B11" t="s">
         <v>495</v>
-      </c>
-      <c r="B11" t="s">
-        <v>496</v>
       </c>
       <c r="C11" t="s">
         <v>5</v>
@@ -5398,66 +5387,66 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>496</v>
+      </c>
+      <c r="B12" t="s">
         <v>497</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>498</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>499</v>
-      </c>
-      <c r="D12" t="s">
-        <v>500</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>500</v>
+      </c>
+      <c r="B13" t="s">
         <v>501</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>502</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>503</v>
-      </c>
-      <c r="D13" t="s">
-        <v>504</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>504</v>
+      </c>
+      <c r="B14" t="s">
         <v>505</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>506</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>507</v>
-      </c>
-      <c r="D14" t="s">
-        <v>508</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>508</v>
+      </c>
+      <c r="B15" t="s">
         <v>509</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>510</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>511</v>
-      </c>
-      <c r="D15" t="s">
-        <v>512</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>512</v>
+      </c>
+      <c r="B16" t="s">
         <v>513</v>
-      </c>
-      <c r="B16" t="s">
-        <v>514</v>
       </c>
       <c r="C16" t="s">
         <v>5</v>
@@ -5468,80 +5457,80 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>514</v>
+      </c>
+      <c r="B17" t="s">
         <v>515</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>516</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>517</v>
-      </c>
-      <c r="D17" t="s">
-        <v>518</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>518</v>
+      </c>
+      <c r="B18" t="s">
         <v>519</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>520</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>521</v>
-      </c>
-      <c r="D18" t="s">
-        <v>522</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>522</v>
+      </c>
+      <c r="B19" t="s">
         <v>523</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>524</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>525</v>
-      </c>
-      <c r="D19" t="s">
-        <v>526</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>526</v>
+      </c>
+      <c r="B20" t="s">
         <v>527</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>528</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>529</v>
-      </c>
-      <c r="D20" t="s">
-        <v>530</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>530</v>
+      </c>
+      <c r="B21" t="s">
         <v>531</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
         <v>532</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>533</v>
-      </c>
-      <c r="D21" t="s">
-        <v>534</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>534</v>
+      </c>
+      <c r="B22" t="s">
         <v>535</v>
-      </c>
-      <c r="B22" t="s">
-        <v>536</v>
       </c>
       <c r="C22" t="s">
         <v>5</v>
@@ -5552,10 +5541,10 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>536</v>
+      </c>
+      <c r="B23" t="s">
         <v>537</v>
-      </c>
-      <c r="B23" t="s">
-        <v>538</v>
       </c>
       <c r="C23" t="s">
         <v>5</v>
@@ -5566,10 +5555,10 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>538</v>
+      </c>
+      <c r="B24" t="s">
         <v>539</v>
-      </c>
-      <c r="B24" t="s">
-        <v>540</v>
       </c>
       <c r="C24" t="s">
         <v>5</v>
@@ -5580,10 +5569,10 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>540</v>
+      </c>
+      <c r="B25" t="s">
         <v>541</v>
-      </c>
-      <c r="B25" t="s">
-        <v>542</v>
       </c>
       <c r="C25" t="s">
         <v>5</v>
@@ -5594,27 +5583,27 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>542</v>
+      </c>
+      <c r="B26" t="s">
         <v>543</v>
       </c>
-      <c r="B26" t="s">
+      <c r="C26" t="s">
         <v>544</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
         <v>545</v>
-      </c>
-      <c r="D26" t="s">
-        <v>546</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>546</v>
+      </c>
+      <c r="B27" t="s">
         <v>547</v>
       </c>
-      <c r="B27" t="s">
+      <c r="C27" t="s">
         <v>548</v>
-      </c>
-      <c r="C27" t="s">
-        <v>549</v>
       </c>
       <c r="D27" t="s">
         <v>5</v>
@@ -5622,10 +5611,10 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>549</v>
+      </c>
+      <c r="B28" t="s">
         <v>550</v>
-      </c>
-      <c r="B28" t="s">
-        <v>551</v>
       </c>
       <c r="C28" t="s">
         <v>5</v>
@@ -5636,10 +5625,10 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>551</v>
+      </c>
+      <c r="B29" t="s">
         <v>552</v>
-      </c>
-      <c r="B29" t="s">
-        <v>553</v>
       </c>
       <c r="C29" t="s">
         <v>5</v>
@@ -5650,10 +5639,10 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>553</v>
+      </c>
+      <c r="B30" t="s">
         <v>554</v>
-      </c>
-      <c r="B30" t="s">
-        <v>555</v>
       </c>
       <c r="C30" t="s">
         <v>5</v>
@@ -5664,27 +5653,27 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>555</v>
+      </c>
+      <c r="B31" t="s">
         <v>556</v>
       </c>
-      <c r="B31" t="s">
+      <c r="C31" t="s">
         <v>557</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
         <v>558</v>
-      </c>
-      <c r="D31" t="s">
-        <v>559</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>559</v>
+      </c>
+      <c r="B32" t="s">
         <v>560</v>
       </c>
-      <c r="B32" t="s">
+      <c r="C32" t="s">
         <v>561</v>
-      </c>
-      <c r="C32" t="s">
-        <v>562</v>
       </c>
       <c r="D32" t="s">
         <v>5</v>
@@ -5692,24 +5681,24 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>562</v>
+      </c>
+      <c r="B33" t="s">
         <v>563</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
         <v>564</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
         <v>565</v>
-      </c>
-      <c r="D33" t="s">
-        <v>566</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>566</v>
+      </c>
+      <c r="B34" t="s">
         <v>567</v>
-      </c>
-      <c r="B34" t="s">
-        <v>568</v>
       </c>
       <c r="C34" t="s">
         <v>5</v>
@@ -5720,10 +5709,10 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>568</v>
+      </c>
+      <c r="B35" t="s">
         <v>569</v>
-      </c>
-      <c r="B35" t="s">
-        <v>570</v>
       </c>
       <c r="C35" t="s">
         <v>5</v>
@@ -5734,10 +5723,10 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>570</v>
+      </c>
+      <c r="B36" t="s">
         <v>571</v>
-      </c>
-      <c r="B36" t="s">
-        <v>572</v>
       </c>
       <c r="C36" t="s">
         <v>5</v>
@@ -5748,10 +5737,10 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>572</v>
+      </c>
+      <c r="B37" t="s">
         <v>573</v>
-      </c>
-      <c r="B37" t="s">
-        <v>574</v>
       </c>
       <c r="C37" t="s">
         <v>5</v>
@@ -5762,10 +5751,10 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>574</v>
+      </c>
+      <c r="B38" t="s">
         <v>575</v>
-      </c>
-      <c r="B38" t="s">
-        <v>576</v>
       </c>
       <c r="C38" t="s">
         <v>5</v>
@@ -5776,10 +5765,10 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>576</v>
+      </c>
+      <c r="B39" t="s">
         <v>577</v>
-      </c>
-      <c r="B39" t="s">
-        <v>578</v>
       </c>
       <c r="C39" t="s">
         <v>5</v>
@@ -5790,10 +5779,10 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>578</v>
+      </c>
+      <c r="B40" t="s">
         <v>579</v>
-      </c>
-      <c r="B40" t="s">
-        <v>580</v>
       </c>
       <c r="C40" t="s">
         <v>5</v>
@@ -5804,10 +5793,10 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>580</v>
+      </c>
+      <c r="B41" t="s">
         <v>581</v>
-      </c>
-      <c r="B41" t="s">
-        <v>582</v>
       </c>
       <c r="C41" t="s">
         <v>5</v>
@@ -5818,24 +5807,24 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>582</v>
+      </c>
+      <c r="B42" t="s">
         <v>583</v>
       </c>
-      <c r="B42" t="s">
+      <c r="C42" t="s">
         <v>584</v>
       </c>
-      <c r="C42" t="s">
+      <c r="D42" t="s">
         <v>585</v>
-      </c>
-      <c r="D42" t="s">
-        <v>586</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>586</v>
+      </c>
+      <c r="B43" t="s">
         <v>587</v>
-      </c>
-      <c r="B43" t="s">
-        <v>588</v>
       </c>
       <c r="C43" t="s">
         <v>5</v>
@@ -5846,10 +5835,10 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>588</v>
+      </c>
+      <c r="B44" t="s">
         <v>589</v>
-      </c>
-      <c r="B44" t="s">
-        <v>590</v>
       </c>
       <c r="C44" t="s">
         <v>5</v>
@@ -5860,10 +5849,10 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
+        <v>590</v>
+      </c>
+      <c r="B45" t="s">
         <v>591</v>
-      </c>
-      <c r="B45" t="s">
-        <v>592</v>
       </c>
       <c r="C45" t="s">
         <v>5</v>
@@ -5874,10 +5863,10 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>592</v>
+      </c>
+      <c r="B46" t="s">
         <v>593</v>
-      </c>
-      <c r="B46" t="s">
-        <v>594</v>
       </c>
       <c r="C46" t="s">
         <v>5</v>
@@ -5888,10 +5877,10 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
+        <v>594</v>
+      </c>
+      <c r="B47" t="s">
         <v>595</v>
-      </c>
-      <c r="B47" t="s">
-        <v>596</v>
       </c>
       <c r="C47" t="s">
         <v>5</v>
@@ -5902,24 +5891,24 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>596</v>
+      </c>
+      <c r="B48" t="s">
         <v>597</v>
       </c>
-      <c r="B48" t="s">
+      <c r="C48" t="s">
         <v>598</v>
       </c>
-      <c r="C48" t="s">
+      <c r="D48" t="s">
         <v>599</v>
-      </c>
-      <c r="D48" t="s">
-        <v>600</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>600</v>
+      </c>
+      <c r="B49" t="s">
         <v>601</v>
-      </c>
-      <c r="B49" t="s">
-        <v>602</v>
       </c>
       <c r="C49" t="s">
         <v>5</v>
@@ -5930,24 +5919,24 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>602</v>
+      </c>
+      <c r="B50" t="s">
         <v>603</v>
       </c>
-      <c r="B50" t="s">
+      <c r="C50" t="s">
         <v>604</v>
       </c>
-      <c r="C50" t="s">
+      <c r="D50" t="s">
         <v>605</v>
-      </c>
-      <c r="D50" t="s">
-        <v>606</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>606</v>
+      </c>
+      <c r="B51" t="s">
         <v>607</v>
-      </c>
-      <c r="B51" t="s">
-        <v>608</v>
       </c>
       <c r="C51" t="s">
         <v>5</v>
@@ -5958,24 +5947,24 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>608</v>
+      </c>
+      <c r="B52" t="s">
         <v>609</v>
       </c>
-      <c r="B52" t="s">
+      <c r="C52" t="s">
         <v>610</v>
       </c>
-      <c r="C52" t="s">
+      <c r="D52" t="s">
         <v>611</v>
-      </c>
-      <c r="D52" t="s">
-        <v>612</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>612</v>
+      </c>
+      <c r="B53" t="s">
         <v>613</v>
-      </c>
-      <c r="B53" t="s">
-        <v>614</v>
       </c>
       <c r="C53" t="s">
         <v>5</v>
@@ -5986,24 +5975,24 @@
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>614</v>
+      </c>
+      <c r="B54" t="s">
         <v>615</v>
       </c>
-      <c r="B54" t="s">
+      <c r="C54" t="s">
         <v>616</v>
       </c>
-      <c r="C54" t="s">
+      <c r="D54" t="s">
         <v>617</v>
-      </c>
-      <c r="D54" t="s">
-        <v>618</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>618</v>
+      </c>
+      <c r="B55" t="s">
         <v>619</v>
-      </c>
-      <c r="B55" t="s">
-        <v>620</v>
       </c>
       <c r="C55" t="s">
         <v>5</v>
@@ -6014,16 +6003,16 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>5</v>
+        <v>884</v>
       </c>
       <c r="B56" t="s">
+        <v>620</v>
+      </c>
+      <c r="C56" t="s">
         <v>621</v>
       </c>
-      <c r="C56" t="s">
+      <c r="D56" t="s">
         <v>622</v>
-      </c>
-      <c r="D56" t="s">
-        <v>623</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -6031,19 +6020,19 @@
         <v>5</v>
       </c>
       <c r="B57" t="s">
+        <v>623</v>
+      </c>
+      <c r="C57" t="s">
         <v>624</v>
       </c>
-      <c r="C57" t="s">
+      <c r="D57" t="s">
         <v>625</v>
-      </c>
-      <c r="D57" t="s">
-        <v>626</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:D57" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:D55 A57:D57 B56:D56" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6070,10 +6059,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>626</v>
+      </c>
+      <c r="B2" t="s">
         <v>627</v>
-      </c>
-      <c r="B2" t="s">
-        <v>628</v>
       </c>
       <c r="C2" t="s">
         <v>5</v>
@@ -6081,21 +6070,21 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>628</v>
+      </c>
+      <c r="B3" t="s">
         <v>629</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>630</v>
-      </c>
-      <c r="C3" t="s">
-        <v>631</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>631</v>
+      </c>
+      <c r="B4" t="s">
         <v>632</v>
-      </c>
-      <c r="B4" t="s">
-        <v>633</v>
       </c>
       <c r="C4" t="s">
         <v>5</v>
@@ -6103,54 +6092,54 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>633</v>
+      </c>
+      <c r="B5" t="s">
         <v>634</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>635</v>
-      </c>
-      <c r="C5" t="s">
-        <v>636</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="B6" t="s">
+        <v>636</v>
+      </c>
+      <c r="C6" t="s">
         <v>637</v>
-      </c>
-      <c r="C6" t="s">
-        <v>638</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>638</v>
+      </c>
+      <c r="B7" t="s">
         <v>639</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>640</v>
-      </c>
-      <c r="C7" t="s">
-        <v>641</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>641</v>
+      </c>
+      <c r="B8" t="s">
         <v>642</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>643</v>
-      </c>
-      <c r="C8" t="s">
-        <v>644</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>644</v>
+      </c>
+      <c r="B9" t="s">
         <v>645</v>
-      </c>
-      <c r="B9" t="s">
-        <v>646</v>
       </c>
       <c r="C9" t="s">
         <v>5</v>
@@ -6158,87 +6147,87 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>646</v>
+      </c>
+      <c r="B10" t="s">
         <v>647</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>648</v>
-      </c>
-      <c r="C10" t="s">
-        <v>649</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>649</v>
+      </c>
+      <c r="B11" t="s">
         <v>650</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>651</v>
-      </c>
-      <c r="C11" t="s">
-        <v>652</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>652</v>
+      </c>
+      <c r="B12" t="s">
         <v>653</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>654</v>
-      </c>
-      <c r="C12" t="s">
-        <v>655</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>655</v>
+      </c>
+      <c r="B13" t="s">
         <v>656</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>657</v>
-      </c>
-      <c r="C13" t="s">
-        <v>658</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>658</v>
+      </c>
+      <c r="B14" t="s">
         <v>659</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>660</v>
-      </c>
-      <c r="C14" t="s">
-        <v>661</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>661</v>
+      </c>
+      <c r="B15" t="s">
         <v>662</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>663</v>
-      </c>
-      <c r="C15" t="s">
-        <v>664</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>664</v>
+      </c>
+      <c r="B16" t="s">
         <v>665</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>666</v>
-      </c>
-      <c r="C16" t="s">
-        <v>667</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>667</v>
+      </c>
+      <c r="B17" t="s">
         <v>668</v>
-      </c>
-      <c r="B17" t="s">
-        <v>669</v>
       </c>
       <c r="C17" t="s">
         <v>5</v>
@@ -6246,10 +6235,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>669</v>
+      </c>
+      <c r="B18" t="s">
         <v>670</v>
-      </c>
-      <c r="B18" t="s">
-        <v>671</v>
       </c>
       <c r="C18" t="s">
         <v>5</v>
@@ -6257,21 +6246,21 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>671</v>
+      </c>
+      <c r="B19" t="s">
         <v>672</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>673</v>
-      </c>
-      <c r="C19" t="s">
-        <v>674</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>674</v>
+      </c>
+      <c r="B20" t="s">
         <v>675</v>
-      </c>
-      <c r="B20" t="s">
-        <v>676</v>
       </c>
       <c r="C20" t="s">
         <v>5</v>
@@ -6279,120 +6268,120 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>676</v>
+      </c>
+      <c r="B21" t="s">
         <v>677</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
         <v>678</v>
-      </c>
-      <c r="C21" t="s">
-        <v>679</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>679</v>
+      </c>
+      <c r="B22" t="s">
         <v>680</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
         <v>681</v>
-      </c>
-      <c r="C22" t="s">
-        <v>682</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>682</v>
+      </c>
+      <c r="B23" t="s">
         <v>683</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" t="s">
         <v>684</v>
-      </c>
-      <c r="C23" t="s">
-        <v>685</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>685</v>
+      </c>
+      <c r="B24" t="s">
         <v>686</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>687</v>
-      </c>
-      <c r="C24" t="s">
-        <v>688</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>688</v>
+      </c>
+      <c r="B25" t="s">
         <v>689</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
         <v>690</v>
-      </c>
-      <c r="C25" t="s">
-        <v>691</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>691</v>
+      </c>
+      <c r="B26" t="s">
         <v>692</v>
       </c>
-      <c r="B26" t="s">
+      <c r="C26" t="s">
         <v>693</v>
-      </c>
-      <c r="C26" t="s">
-        <v>694</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>694</v>
+      </c>
+      <c r="B27" t="s">
         <v>695</v>
       </c>
-      <c r="B27" t="s">
+      <c r="C27" t="s">
         <v>696</v>
-      </c>
-      <c r="C27" t="s">
-        <v>697</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>697</v>
+      </c>
+      <c r="B28" t="s">
         <v>698</v>
       </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
         <v>699</v>
-      </c>
-      <c r="C28" t="s">
-        <v>700</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>700</v>
+      </c>
+      <c r="B29" t="s">
         <v>701</v>
       </c>
-      <c r="B29" t="s">
+      <c r="C29" t="s">
         <v>702</v>
-      </c>
-      <c r="C29" t="s">
-        <v>703</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>703</v>
+      </c>
+      <c r="B30" t="s">
         <v>704</v>
       </c>
-      <c r="B30" t="s">
+      <c r="C30" t="s">
         <v>705</v>
-      </c>
-      <c r="C30" t="s">
-        <v>706</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>706</v>
+      </c>
+      <c r="B31" t="s">
         <v>707</v>
-      </c>
-      <c r="B31" t="s">
-        <v>708</v>
       </c>
       <c r="C31" t="s">
         <v>5</v>
@@ -6400,98 +6389,98 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>708</v>
+      </c>
+      <c r="B32" t="s">
         <v>709</v>
       </c>
-      <c r="B32" t="s">
+      <c r="C32" t="s">
         <v>710</v>
-      </c>
-      <c r="C32" t="s">
-        <v>711</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>711</v>
+      </c>
+      <c r="B33" t="s">
         <v>712</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
         <v>713</v>
-      </c>
-      <c r="C33" t="s">
-        <v>714</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>714</v>
+      </c>
+      <c r="B34" t="s">
         <v>715</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" t="s">
         <v>716</v>
-      </c>
-      <c r="C34" t="s">
-        <v>717</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>717</v>
+      </c>
+      <c r="B35" t="s">
         <v>718</v>
       </c>
-      <c r="B35" t="s">
+      <c r="C35" t="s">
         <v>719</v>
-      </c>
-      <c r="C35" t="s">
-        <v>720</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>720</v>
+      </c>
+      <c r="B36" t="s">
         <v>721</v>
       </c>
-      <c r="B36" t="s">
+      <c r="C36" t="s">
         <v>722</v>
-      </c>
-      <c r="C36" t="s">
-        <v>723</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>723</v>
+      </c>
+      <c r="B37" t="s">
         <v>724</v>
       </c>
-      <c r="B37" t="s">
+      <c r="C37" t="s">
         <v>725</v>
-      </c>
-      <c r="C37" t="s">
-        <v>726</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>726</v>
+      </c>
+      <c r="B38" t="s">
         <v>727</v>
       </c>
-      <c r="B38" t="s">
+      <c r="C38" t="s">
         <v>728</v>
-      </c>
-      <c r="C38" t="s">
-        <v>729</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>729</v>
+      </c>
+      <c r="B39" t="s">
         <v>730</v>
       </c>
-      <c r="B39" t="s">
+      <c r="C39" t="s">
         <v>731</v>
-      </c>
-      <c r="C39" t="s">
-        <v>732</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>732</v>
+      </c>
+      <c r="B40" t="s">
         <v>733</v>
-      </c>
-      <c r="B40" t="s">
-        <v>734</v>
       </c>
       <c r="C40" t="s">
         <v>5</v>
@@ -6499,10 +6488,10 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>734</v>
+      </c>
+      <c r="B41" t="s">
         <v>735</v>
-      </c>
-      <c r="B41" t="s">
-        <v>736</v>
       </c>
       <c r="C41" t="s">
         <v>5</v>
@@ -6510,285 +6499,285 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>736</v>
+      </c>
+      <c r="B42" t="s">
         <v>737</v>
       </c>
-      <c r="B42" t="s">
+      <c r="C42" t="s">
         <v>738</v>
-      </c>
-      <c r="C42" t="s">
-        <v>739</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>739</v>
+      </c>
+      <c r="B43" t="s">
         <v>740</v>
       </c>
-      <c r="B43" t="s">
+      <c r="C43" t="s">
         <v>741</v>
-      </c>
-      <c r="C43" t="s">
-        <v>742</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>742</v>
+      </c>
+      <c r="B44" t="s">
         <v>743</v>
       </c>
-      <c r="B44" t="s">
+      <c r="C44" t="s">
         <v>744</v>
-      </c>
-      <c r="C44" t="s">
-        <v>745</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
+        <v>745</v>
+      </c>
+      <c r="B45" t="s">
         <v>746</v>
       </c>
-      <c r="B45" t="s">
+      <c r="C45" t="s">
         <v>747</v>
-      </c>
-      <c r="C45" t="s">
-        <v>748</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>748</v>
+      </c>
+      <c r="B46" t="s">
         <v>749</v>
       </c>
-      <c r="B46" t="s">
+      <c r="C46" t="s">
         <v>750</v>
-      </c>
-      <c r="C46" t="s">
-        <v>751</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
+        <v>751</v>
+      </c>
+      <c r="B47" t="s">
         <v>752</v>
       </c>
-      <c r="B47" t="s">
+      <c r="C47" t="s">
         <v>753</v>
-      </c>
-      <c r="C47" t="s">
-        <v>754</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="B48" t="s">
+        <v>882</v>
+      </c>
+      <c r="C48" s="1" t="s">
         <v>883</v>
-      </c>
-      <c r="C48" s="1" t="s">
-        <v>884</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>755</v>
+      </c>
+      <c r="B49" t="s">
         <v>756</v>
       </c>
-      <c r="B49" t="s">
+      <c r="C49" t="s">
         <v>757</v>
-      </c>
-      <c r="C49" t="s">
-        <v>758</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>758</v>
+      </c>
+      <c r="B50" t="s">
         <v>759</v>
       </c>
-      <c r="B50" t="s">
+      <c r="C50" t="s">
         <v>760</v>
-      </c>
-      <c r="C50" t="s">
-        <v>761</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>761</v>
+      </c>
+      <c r="B51" t="s">
         <v>762</v>
       </c>
-      <c r="B51" t="s">
+      <c r="C51" t="s">
         <v>763</v>
-      </c>
-      <c r="C51" t="s">
-        <v>764</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>764</v>
+      </c>
+      <c r="B52" t="s">
         <v>765</v>
       </c>
-      <c r="B52" t="s">
+      <c r="C52" t="s">
         <v>766</v>
-      </c>
-      <c r="C52" t="s">
-        <v>767</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>767</v>
+      </c>
+      <c r="B53" t="s">
         <v>768</v>
       </c>
-      <c r="B53" t="s">
+      <c r="C53" t="s">
         <v>769</v>
-      </c>
-      <c r="C53" t="s">
-        <v>770</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>770</v>
+      </c>
+      <c r="B54" t="s">
         <v>771</v>
       </c>
-      <c r="B54" t="s">
+      <c r="C54" t="s">
         <v>772</v>
-      </c>
-      <c r="C54" t="s">
-        <v>773</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>773</v>
+      </c>
+      <c r="B55" t="s">
         <v>774</v>
       </c>
-      <c r="B55" t="s">
+      <c r="C55" t="s">
         <v>775</v>
-      </c>
-      <c r="C55" t="s">
-        <v>776</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>776</v>
+      </c>
+      <c r="B56" t="s">
         <v>777</v>
       </c>
-      <c r="B56" t="s">
+      <c r="C56" t="s">
         <v>778</v>
-      </c>
-      <c r="C56" t="s">
-        <v>779</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
+        <v>779</v>
+      </c>
+      <c r="B57" t="s">
         <v>780</v>
       </c>
-      <c r="B57" t="s">
+      <c r="C57" t="s">
         <v>781</v>
-      </c>
-      <c r="C57" t="s">
-        <v>782</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
+        <v>782</v>
+      </c>
+      <c r="B58" t="s">
         <v>783</v>
       </c>
-      <c r="B58" t="s">
+      <c r="C58" t="s">
         <v>784</v>
-      </c>
-      <c r="C58" t="s">
-        <v>785</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
+        <v>785</v>
+      </c>
+      <c r="B59" t="s">
         <v>786</v>
       </c>
-      <c r="B59" t="s">
+      <c r="C59" t="s">
         <v>787</v>
-      </c>
-      <c r="C59" t="s">
-        <v>788</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>788</v>
+      </c>
+      <c r="B60" t="s">
         <v>789</v>
       </c>
-      <c r="B60" t="s">
+      <c r="C60" t="s">
         <v>790</v>
-      </c>
-      <c r="C60" t="s">
-        <v>791</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
+        <v>791</v>
+      </c>
+      <c r="B61" t="s">
         <v>792</v>
       </c>
-      <c r="B61" t="s">
+      <c r="C61" t="s">
         <v>793</v>
-      </c>
-      <c r="C61" t="s">
-        <v>794</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
+        <v>794</v>
+      </c>
+      <c r="B62" t="s">
         <v>795</v>
       </c>
-      <c r="B62" t="s">
+      <c r="C62" t="s">
         <v>796</v>
-      </c>
-      <c r="C62" t="s">
-        <v>797</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
+        <v>797</v>
+      </c>
+      <c r="B63" t="s">
         <v>798</v>
       </c>
-      <c r="B63" t="s">
+      <c r="C63" t="s">
         <v>799</v>
-      </c>
-      <c r="C63" t="s">
-        <v>800</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>800</v>
+      </c>
+      <c r="B64" t="s">
         <v>801</v>
       </c>
-      <c r="B64" t="s">
+      <c r="C64" t="s">
         <v>802</v>
-      </c>
-      <c r="C64" t="s">
-        <v>803</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>803</v>
+      </c>
+      <c r="B65" t="s">
         <v>804</v>
       </c>
-      <c r="B65" t="s">
+      <c r="C65" t="s">
         <v>805</v>
-      </c>
-      <c r="C65" t="s">
-        <v>806</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
+        <v>806</v>
+      </c>
+      <c r="B66" t="s">
         <v>807</v>
       </c>
-      <c r="B66" t="s">
+      <c r="C66" t="s">
         <v>808</v>
-      </c>
-      <c r="C66" t="s">
-        <v>809</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
+        <v>809</v>
+      </c>
+      <c r="B67" t="s">
         <v>810</v>
-      </c>
-      <c r="B67" t="s">
-        <v>811</v>
       </c>
       <c r="C67" t="s">
         <v>5</v>
@@ -6796,43 +6785,43 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>811</v>
+      </c>
+      <c r="B68" t="s">
         <v>812</v>
       </c>
-      <c r="B68" t="s">
+      <c r="C68" t="s">
         <v>813</v>
-      </c>
-      <c r="C68" t="s">
-        <v>814</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
+        <v>814</v>
+      </c>
+      <c r="B69" t="s">
         <v>815</v>
       </c>
-      <c r="B69" t="s">
+      <c r="C69" t="s">
         <v>816</v>
-      </c>
-      <c r="C69" t="s">
-        <v>817</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>817</v>
+      </c>
+      <c r="B70" t="s">
         <v>818</v>
       </c>
-      <c r="B70" t="s">
+      <c r="C70" t="s">
         <v>819</v>
-      </c>
-      <c r="C70" t="s">
-        <v>820</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
+        <v>820</v>
+      </c>
+      <c r="B71" t="s">
         <v>821</v>
-      </c>
-      <c r="B71" t="s">
-        <v>822</v>
       </c>
       <c r="C71" t="s">
         <v>5</v>
@@ -6840,10 +6829,10 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
+        <v>822</v>
+      </c>
+      <c r="B72" t="s">
         <v>823</v>
-      </c>
-      <c r="B72" t="s">
-        <v>824</v>
       </c>
       <c r="C72" t="s">
         <v>5</v>
@@ -6851,10 +6840,10 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
+        <v>824</v>
+      </c>
+      <c r="B73" t="s">
         <v>825</v>
-      </c>
-      <c r="B73" t="s">
-        <v>826</v>
       </c>
       <c r="C73" t="s">
         <v>5</v>
@@ -6865,7 +6854,7 @@
         <v>271</v>
       </c>
       <c r="B74" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="C74" t="s">
         <v>273</v>
@@ -6873,10 +6862,10 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
+        <v>827</v>
+      </c>
+      <c r="B75" t="s">
         <v>828</v>
-      </c>
-      <c r="B75" t="s">
-        <v>829</v>
       </c>
       <c r="C75" t="s">
         <v>5</v>
@@ -6884,43 +6873,43 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
+        <v>829</v>
+      </c>
+      <c r="B76" t="s">
         <v>830</v>
       </c>
-      <c r="B76" t="s">
+      <c r="C76" t="s">
         <v>831</v>
-      </c>
-      <c r="C76" t="s">
-        <v>832</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
+        <v>832</v>
+      </c>
+      <c r="B77" t="s">
         <v>833</v>
       </c>
-      <c r="B77" t="s">
+      <c r="C77" t="s">
         <v>834</v>
-      </c>
-      <c r="C77" t="s">
-        <v>835</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
+        <v>835</v>
+      </c>
+      <c r="B78" t="s">
         <v>836</v>
       </c>
-      <c r="B78" t="s">
+      <c r="C78" t="s">
         <v>837</v>
-      </c>
-      <c r="C78" t="s">
-        <v>838</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
+        <v>838</v>
+      </c>
+      <c r="B79" t="s">
         <v>839</v>
-      </c>
-      <c r="B79" t="s">
-        <v>840</v>
       </c>
       <c r="C79" t="s">
         <v>5</v>
@@ -6928,21 +6917,21 @@
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
+        <v>840</v>
+      </c>
+      <c r="B80" t="s">
         <v>841</v>
       </c>
-      <c r="B80" t="s">
+      <c r="C80" t="s">
         <v>842</v>
-      </c>
-      <c r="C80" t="s">
-        <v>843</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
+        <v>843</v>
+      </c>
+      <c r="B81" t="s">
         <v>844</v>
-      </c>
-      <c r="B81" t="s">
-        <v>845</v>
       </c>
       <c r="C81" t="s">
         <v>5</v>
@@ -6950,21 +6939,21 @@
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>845</v>
+      </c>
+      <c r="B82" t="s">
         <v>846</v>
       </c>
-      <c r="B82" t="s">
+      <c r="C82" t="s">
         <v>847</v>
-      </c>
-      <c r="C82" t="s">
-        <v>848</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
+        <v>848</v>
+      </c>
+      <c r="B83" t="s">
         <v>849</v>
-      </c>
-      <c r="B83" t="s">
-        <v>850</v>
       </c>
       <c r="C83" t="s">
         <v>5</v>
@@ -6972,21 +6961,21 @@
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
+        <v>850</v>
+      </c>
+      <c r="B84" t="s">
         <v>851</v>
       </c>
-      <c r="B84" t="s">
+      <c r="C84" t="s">
         <v>852</v>
-      </c>
-      <c r="C84" t="s">
-        <v>853</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
+        <v>853</v>
+      </c>
+      <c r="B85" t="s">
         <v>854</v>
-      </c>
-      <c r="B85" t="s">
-        <v>855</v>
       </c>
       <c r="C85" t="s">
         <v>5</v>
@@ -6994,10 +6983,10 @@
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
+        <v>855</v>
+      </c>
+      <c r="B86" t="s">
         <v>856</v>
-      </c>
-      <c r="B86" t="s">
-        <v>857</v>
       </c>
       <c r="C86" t="s">
         <v>5</v>
@@ -7005,79 +6994,79 @@
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
+        <v>857</v>
+      </c>
+      <c r="B87" t="s">
         <v>858</v>
       </c>
-      <c r="B87" t="s">
+      <c r="C87" t="s">
         <v>859</v>
-      </c>
-      <c r="C87" t="s">
-        <v>860</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="B88" t="s">
+        <v>672</v>
+      </c>
+      <c r="C88" t="s">
         <v>673</v>
-      </c>
-      <c r="C88" t="s">
-        <v>674</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
+        <v>861</v>
+      </c>
+      <c r="B89" t="s">
         <v>862</v>
       </c>
-      <c r="B89" t="s">
+      <c r="C89" t="s">
         <v>863</v>
-      </c>
-      <c r="C89" t="s">
-        <v>864</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
+        <v>864</v>
+      </c>
+      <c r="B90" t="s">
         <v>865</v>
       </c>
-      <c r="B90" t="s">
+      <c r="C90" t="s">
         <v>866</v>
-      </c>
-      <c r="C90" t="s">
-        <v>867</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
+        <v>867</v>
+      </c>
+      <c r="B91" t="s">
         <v>868</v>
       </c>
-      <c r="B91" t="s">
+      <c r="C91" t="s">
         <v>869</v>
-      </c>
-      <c r="C91" t="s">
-        <v>870</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
+        <v>870</v>
+      </c>
+      <c r="B92" t="s">
         <v>871</v>
       </c>
-      <c r="B92" t="s">
+      <c r="C92" t="s">
         <v>872</v>
-      </c>
-      <c r="C92" t="s">
-        <v>873</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
+        <v>873</v>
+      </c>
+      <c r="B93" t="s">
         <v>874</v>
       </c>
-      <c r="B93" t="s">
+      <c r="C93" t="s">
         <v>875</v>
-      </c>
-      <c r="C93" t="s">
-        <v>876</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
@@ -7085,21 +7074,21 @@
         <v>267</v>
       </c>
       <c r="B94" t="s">
+        <v>876</v>
+      </c>
+      <c r="C94" t="s">
         <v>877</v>
-      </c>
-      <c r="C94" t="s">
-        <v>878</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="B95" t="s">
+        <v>878</v>
+      </c>
+      <c r="C95" t="s">
         <v>879</v>
-      </c>
-      <c r="C95" t="s">
-        <v>880</v>
       </c>
     </row>
   </sheetData>

</xml_diff>